<commit_message>
feat: Remplacement de l'apercu Excel par le PDF natif
</commit_message>
<xml_diff>
--- a/Tableau de synthèse.xlsx
+++ b/Tableau de synthèse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Portfolio-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{486B5F41-72C9-4550-9F70-64B370C23BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72FE275-D234-41BA-85AD-DD5ED5094523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -89,9 +89,6 @@
     <t>▢ SISR</t>
   </si>
   <si>
-    <t>▢ SLAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Réalisation en cours de formation
 </t>
   </si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>Projet de développement d'une interface graphique avec Vue.JS pour orchestrer des modèles d'IA (Ollama) capables d'interagir avec le système d'exploitation pour effectuer des audits réseau avec Nmap.</t>
+  </si>
+  <si>
+    <t>☒ SLAM</t>
   </si>
 </sst>
 </file>
@@ -701,6 +701,33 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -716,9 +743,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -750,30 +774,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1095,56 +1095,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="31"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="G3" s="44"/>
-      <c r="H3" s="50"/>
+      <c r="A3" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="28"/>
+      <c r="H3" s="34"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="48"/>
+      <c r="A4" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
       <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
@@ -1152,27 +1152,27 @@
         <v>15</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="A5" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="50"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="46" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1194,8 +1194,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="30"/>
-      <c r="B7" s="39"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="47"/>
       <c r="C7" s="25" t="s">
         <v>9</v>
       </c>
@@ -1251,16 +1251,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="A8" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1299,10 +1299,10 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
@@ -1348,7 +1348,7 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="23">
         <v>45748</v>
@@ -1397,7 +1397,7 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="22">
         <v>45734</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="22">
         <v>45646</v>
@@ -1495,7 +1495,7 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="22">
         <v>45734</v>
@@ -1544,7 +1544,7 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="23">
         <v>45627</v>
@@ -1593,7 +1593,7 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="22">
         <v>45758</v>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="22">
         <v>45646</v>
@@ -1691,7 +1691,7 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B17" s="22">
         <v>45741</v>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="22">
         <v>45779</v>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
@@ -1838,10 +1838,10 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
@@ -1886,16 +1886,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A21" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="37"/>
+      <c r="A21" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="44"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="45"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1934,10 +1934,10 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
@@ -1982,16 +1982,16 @@
       <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="28"/>
+      <c r="A23" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="37"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2030,10 +2030,10 @@
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
@@ -2128,10 +2128,10 @@
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
@@ -2484,11 +2484,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
@@ -2496,6 +2491,11 @@
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2506,6 +2506,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DB4A65246D1F9A438D5F9AB5F8564BE0" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="0f798571656b0fafde6a2983aa2241aa">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="448e5bc6-220e-4232-be9c-92dc25a4e4e5" xmlns:ns3="2197ab10-882f-4df3-a7c2-cbc9019ef6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdbf8d29756c261afaa0b8b1c078f5c2" ns2:_="" ns3:_="">
     <xsd:import namespace="448e5bc6-220e-4232-be9c-92dc25a4e4e5"/>
@@ -2728,15 +2737,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2749,6 +2749,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCE846E6-82B3-4E26-AE12-6B4ADF4F7EBF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81DD115F-33AC-44C4-851E-680D105EAC1D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2767,14 +2775,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCE846E6-82B3-4E26-AE12-6B4ADF4F7EBF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8699F405-6A98-4E42-A4E6-D622358F7C7F}">
   <ds:schemaRefs>

</xml_diff>